<commit_message>
docs: seguimiento — iteración de PNTs (Markdown + Excel)
</commit_message>
<xml_diff>
--- a/Seguimiento-Paneles-Control.xlsx
+++ b/Seguimiento-Paneles-Control.xlsx
@@ -1575,12 +1575,12 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Bloques PNTs, tabla estilizada, iconos.</t>
+          <t>Tiles de cursos como tarjetas (imagen, badge de plazo, progreso) con filtros y paginación cliente. Filtros como botones azul light; «Curso» en gris (sin azul); badges de plazo con paleta de marca (semáforo teal/ámbar/naranja/rojo + Completado borde navy) y dots de leyenda a juego.</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>CSS secc. 6 (DASHBOARD PNTs) y secc. 20 (BLOQUES PNTs)</t>
+          <t>bloques/3-codigo-actual/pnts-html-adicional.html (JS) · css-totara-organizado.css secc. 6 (DASHBOARD PNTs) y secc. 20 (BLOQUES PNTs)</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1593,7 +1593,11 @@
           <t>☐ Pendiente</t>
         </is>
       </c>
-      <c r="I26" s="5" t="inlineStr"/>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Pendiente purga CDN</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="10" t="inlineStr">

</xml_diff>